<commit_message>
fix: support sheet and header row selection for xlsx uploads
</commit_message>
<xml_diff>
--- a/sample-data/sample_reviews_fashion.xlsx
+++ b/sample-data/sample_reviews_fashion.xlsx
@@ -3,7 +3,10 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="리뷰" sheetId="1" r:id="rId1"/>
+    <sheet name="리뷰데이터" sheetId="1" r:id="rId1"/>
+    <sheet name="오분류_테스트케이스" sheetId="2" r:id="rId2"/>
+    <sheet name="요약" sheetId="3" r:id="rId3"/>
+    <sheet name="README" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I134"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2168,9 +2171,2242 @@
         <v/>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>7001</v>
+      </c>
+      <c r="B62" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C62" t="str">
+        <v>블랙/M</v>
+      </c>
+      <c r="D62" t="str">
+        <v>2</v>
+      </c>
+      <c r="E62" t="str">
+        <v>어깨 좁아요</v>
+      </c>
+      <c r="F62" t="str">
+        <v>오버핏인데 어깨가 좁아서 답답해요. 소매가 너무 길어서 손이 다 가려져요.</v>
+      </c>
+      <c r="G62" t="str">
+        <v>김주원</v>
+      </c>
+      <c r="H62" t="str">
+        <v>2026-05-20</v>
+      </c>
+      <c r="I62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>7002</v>
+      </c>
+      <c r="B63" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C63" t="str">
+        <v>그레이/L</v>
+      </c>
+      <c r="D63" t="str">
+        <v>4</v>
+      </c>
+      <c r="E63" t="str">
+        <v>따뜻해요</v>
+      </c>
+      <c r="F63" t="str">
+        <v>두께감이 적당하고 따뜻해요. 핏도 마음에 들어요. 재구매 의사 있어요.</v>
+      </c>
+      <c r="G63" t="str">
+        <v>이서영</v>
+      </c>
+      <c r="H63" t="str">
+        <v>2026-05-21</v>
+      </c>
+      <c r="I63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>7003</v>
+      </c>
+      <c r="B64" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C64" t="str">
+        <v>블랙/L</v>
+      </c>
+      <c r="D64" t="str">
+        <v>3</v>
+      </c>
+      <c r="E64" t="str">
+        <v>세탁 후 보풀</v>
+      </c>
+      <c r="F64" t="str">
+        <v>한 번 세탁했는데 보풀이 좀 생겼어요. 색상은 사진이랑 비슷합니다.</v>
+      </c>
+      <c r="G64" t="str">
+        <v>박정훈</v>
+      </c>
+      <c r="H64" t="str">
+        <v>2026-05-22</v>
+      </c>
+      <c r="I64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>7004</v>
+      </c>
+      <c r="B65" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C65" t="str">
+        <v>차콜/M</v>
+      </c>
+      <c r="D65" t="str">
+        <v>5</v>
+      </c>
+      <c r="E65" t="str">
+        <v>가성비 굿</v>
+      </c>
+      <c r="F65" t="str">
+        <v>가격에 비해 두께도 좋고 핏도 예뻐요. 강추합니다.</v>
+      </c>
+      <c r="G65" t="str">
+        <v>최승현</v>
+      </c>
+      <c r="H65" t="str">
+        <v>2026-05-23</v>
+      </c>
+      <c r="I65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>7005</v>
+      </c>
+      <c r="B66" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C66" t="str">
+        <v>그레이/L</v>
+      </c>
+      <c r="D66" t="str">
+        <v>2</v>
+      </c>
+      <c r="E66" t="str">
+        <v>소매가 너무 김</v>
+      </c>
+      <c r="F66" t="str">
+        <v>팔이 한참 길어서 접어야 했어요. 키 175인데 소매가 손등 한참 아래까지 옵니다.</v>
+      </c>
+      <c r="G66" t="str">
+        <v>정민혁</v>
+      </c>
+      <c r="H66" t="str">
+        <v>2026-05-24</v>
+      </c>
+      <c r="I66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>7006</v>
+      </c>
+      <c r="B67" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C67" t="str">
+        <v>블랙/M</v>
+      </c>
+      <c r="D67" t="str">
+        <v>4</v>
+      </c>
+      <c r="E67" t="str">
+        <v>편해요</v>
+      </c>
+      <c r="F67" t="str">
+        <v>오버핏 좋아하시면 추천해요. 무게는 살짝 있는 편.</v>
+      </c>
+      <c r="G67" t="str">
+        <v>한가람</v>
+      </c>
+      <c r="H67" t="str">
+        <v>2026-05-25</v>
+      </c>
+      <c r="I67" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>7007</v>
+      </c>
+      <c r="B68" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C68" t="str">
+        <v>차콜/L</v>
+      </c>
+      <c r="D68" t="str">
+        <v>3</v>
+      </c>
+      <c r="E68" t="str">
+        <v>냄새가 좀 나요</v>
+      </c>
+      <c r="F68" t="str">
+        <v>새 제품 특유의 화학약품 냄새가 좀 나요. 며칠 환기하니 사라집니다.</v>
+      </c>
+      <c r="G68" t="str">
+        <v>오지호</v>
+      </c>
+      <c r="H68" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="I68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>7008</v>
+      </c>
+      <c r="B69" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C69" t="str">
+        <v>그레이/M</v>
+      </c>
+      <c r="D69" t="str">
+        <v>5</v>
+      </c>
+      <c r="E69" t="str">
+        <v>재구매 의사</v>
+      </c>
+      <c r="F69" t="str">
+        <v>색상별로 사고 싶을 만큼 만족합니다. 가성비도 좋네요.</v>
+      </c>
+      <c r="G69" t="str">
+        <v>임수정</v>
+      </c>
+      <c r="H69" t="str">
+        <v>2026-05-27</v>
+      </c>
+      <c r="I69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>8001</v>
+      </c>
+      <c r="B70" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C70" t="str">
+        <v>베이지/M</v>
+      </c>
+      <c r="D70" t="str">
+        <v>1</v>
+      </c>
+      <c r="E70" t="str">
+        <v>무겁고 답답해요</v>
+      </c>
+      <c r="F70" t="str">
+        <v>데님보다 무거워서 어깨가 무너지는 느낌이에요. 종일 입고 다니기 힘들었어요.</v>
+      </c>
+      <c r="G70" t="str">
+        <v>김도현</v>
+      </c>
+      <c r="H70" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="I70" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>8002</v>
+      </c>
+      <c r="B71" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C71" t="str">
+        <v>카키/L</v>
+      </c>
+      <c r="D71" t="str">
+        <v>2</v>
+      </c>
+      <c r="E71" t="str">
+        <v>어깨가 좁아요</v>
+      </c>
+      <c r="F71" t="str">
+        <v>어깨가 좁아서 팔 움직이기 불편해요. 한 치수 크게 사세요.</v>
+      </c>
+      <c r="G71" t="str">
+        <v>이혜진</v>
+      </c>
+      <c r="H71" t="str">
+        <v>2026-04-26</v>
+      </c>
+      <c r="I71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>8003</v>
+      </c>
+      <c r="B72" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C72" t="str">
+        <v>블랙/M</v>
+      </c>
+      <c r="D72" t="str">
+        <v>3</v>
+      </c>
+      <c r="E72" t="str">
+        <v>색상 차이</v>
+      </c>
+      <c r="F72" t="str">
+        <v>블랙이라 적었는데 실물은 짙은 회색에 가까워요. 사진이랑 톤이 달라요.</v>
+      </c>
+      <c r="G72" t="str">
+        <v>박상혁</v>
+      </c>
+      <c r="H72" t="str">
+        <v>2026-04-27</v>
+      </c>
+      <c r="I72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>8004</v>
+      </c>
+      <c r="B73" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C73" t="str">
+        <v>베이지/L</v>
+      </c>
+      <c r="D73" t="str">
+        <v>2</v>
+      </c>
+      <c r="E73" t="str">
+        <v>단추 떨어짐</v>
+      </c>
+      <c r="F73" t="str">
+        <v>입은 지 며칠 안 됐는데 단추 하나가 헐거워져서 떨어졌어요. 마감이 아쉽네요.</v>
+      </c>
+      <c r="G73" t="str">
+        <v>최우석</v>
+      </c>
+      <c r="H73" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="I73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>8005</v>
+      </c>
+      <c r="B74" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C74" t="str">
+        <v>카키/M</v>
+      </c>
+      <c r="D74" t="str">
+        <v>4</v>
+      </c>
+      <c r="E74" t="str">
+        <v>핏 예뻐요</v>
+      </c>
+      <c r="F74" t="str">
+        <v>핏 라인이 예쁘게 떨어져요. 다만 두께가 두꺼워서 봄 가을용으로만 입을듯.</v>
+      </c>
+      <c r="G74" t="str">
+        <v>정수민</v>
+      </c>
+      <c r="H74" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="I74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>8006</v>
+      </c>
+      <c r="B75" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C75" t="str">
+        <v>베이지/M</v>
+      </c>
+      <c r="D75" t="str">
+        <v>2</v>
+      </c>
+      <c r="E75" t="str">
+        <v>세탁 후 변형</v>
+      </c>
+      <c r="F75" t="str">
+        <v>드라이만 했는데 어깨 라인이 살짝 틀어졌어요. 세탁 주의가 필요해 보입니다.</v>
+      </c>
+      <c r="G75" t="str">
+        <v>한동훈</v>
+      </c>
+      <c r="H75" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="I75" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>8007</v>
+      </c>
+      <c r="B76" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C76" t="str">
+        <v>블랙/L</v>
+      </c>
+      <c r="D76" t="str">
+        <v>5</v>
+      </c>
+      <c r="E76" t="str">
+        <v>만족해요</v>
+      </c>
+      <c r="F76" t="str">
+        <v>핏도 좋고 무게도 적당해요. 색상 분위기도 좋습니다.</v>
+      </c>
+      <c r="G76" t="str">
+        <v>오민영</v>
+      </c>
+      <c r="H76" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="I76" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>8008</v>
+      </c>
+      <c r="B77" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C77" t="str">
+        <v>카키/L</v>
+      </c>
+      <c r="D77" t="str">
+        <v>2</v>
+      </c>
+      <c r="E77" t="str">
+        <v>보풀과 실밥</v>
+      </c>
+      <c r="F77" t="str">
+        <v>새 옷인데 실밥이 여기저기 튀어나와 있고, 며칠 입으니 보풀도 생겨요.</v>
+      </c>
+      <c r="G77" t="str">
+        <v>신유경</v>
+      </c>
+      <c r="H77" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="I77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>9001</v>
+      </c>
+      <c r="B78" t="str">
+        <v>러닝화</v>
+      </c>
+      <c r="C78" t="str">
+        <v>화이트/270</v>
+      </c>
+      <c r="D78" t="str">
+        <v>1</v>
+      </c>
+      <c r="E78" t="str">
+        <v>사이즈가 작아요</v>
+      </c>
+      <c r="F78" t="str">
+        <v>평소 신던 사이즈 그대로 샀는데 발볼이 좁고 발가락이 끼어요. 한 치수 크게 사세요.</v>
+      </c>
+      <c r="G78" t="str">
+        <v>김건우</v>
+      </c>
+      <c r="H78" t="str">
+        <v>2026-05-05</v>
+      </c>
+      <c r="I78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>9002</v>
+      </c>
+      <c r="B79" t="str">
+        <v>러닝화</v>
+      </c>
+      <c r="C79" t="str">
+        <v>블랙/280</v>
+      </c>
+      <c r="D79" t="str">
+        <v>2</v>
+      </c>
+      <c r="E79" t="str">
+        <v>쿠션감 부족</v>
+      </c>
+      <c r="F79" t="str">
+        <v>러닝화라는데 쿠션감이 별로 없어요. 오래 뛰면 발이 아파요.</v>
+      </c>
+      <c r="G79" t="str">
+        <v>이태경</v>
+      </c>
+      <c r="H79" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="I79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>9003</v>
+      </c>
+      <c r="B80" t="str">
+        <v>러닝화</v>
+      </c>
+      <c r="C80" t="str">
+        <v>그레이/265</v>
+      </c>
+      <c r="D80" t="str">
+        <v>3</v>
+      </c>
+      <c r="E80" t="str">
+        <v>발볼 좁음</v>
+      </c>
+      <c r="F80" t="str">
+        <v>발볼이 좁아서 양말 두꺼운 거 신으면 답답해요. 색상은 사진이랑 비슷합니다.</v>
+      </c>
+      <c r="G80" t="str">
+        <v>박은서</v>
+      </c>
+      <c r="H80" t="str">
+        <v>2026-05-07</v>
+      </c>
+      <c r="I80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>9004</v>
+      </c>
+      <c r="B81" t="str">
+        <v>러닝화</v>
+      </c>
+      <c r="C81" t="str">
+        <v>화이트/275</v>
+      </c>
+      <c r="D81" t="str">
+        <v>2</v>
+      </c>
+      <c r="E81" t="str">
+        <v>뒤꿈치 까져요</v>
+      </c>
+      <c r="F81" t="str">
+        <v>처음 신었을 때 뒤꿈치가 까져서 밴드 붙이고 신었어요. 길들이는 시간이 필요한듯.</v>
+      </c>
+      <c r="G81" t="str">
+        <v>최진우</v>
+      </c>
+      <c r="H81" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="I81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>9005</v>
+      </c>
+      <c r="B82" t="str">
+        <v>러닝화</v>
+      </c>
+      <c r="C82" t="str">
+        <v>블랙/270</v>
+      </c>
+      <c r="D82" t="str">
+        <v>5</v>
+      </c>
+      <c r="E82" t="str">
+        <v>편해요</v>
+      </c>
+      <c r="F82" t="str">
+        <v>가벼워서 산책용으로 좋아요. 가성비 만족합니다.</v>
+      </c>
+      <c r="G82" t="str">
+        <v>정유나</v>
+      </c>
+      <c r="H82" t="str">
+        <v>2026-05-09</v>
+      </c>
+      <c r="I82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>9006</v>
+      </c>
+      <c r="B83" t="str">
+        <v>러닝화</v>
+      </c>
+      <c r="C83" t="str">
+        <v>화이트/280</v>
+      </c>
+      <c r="D83" t="str">
+        <v>2</v>
+      </c>
+      <c r="E83" t="str">
+        <v>배송 늦음</v>
+      </c>
+      <c r="F83" t="str">
+        <v>주문하고 일주일 넘게 늦었어요. 너무 오래 걸렸네요.</v>
+      </c>
+      <c r="G83" t="str">
+        <v>한지영</v>
+      </c>
+      <c r="H83" t="str">
+        <v>2026-05-10</v>
+      </c>
+      <c r="I83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>9007</v>
+      </c>
+      <c r="B84" t="str">
+        <v>러닝화</v>
+      </c>
+      <c r="C84" t="str">
+        <v>그레이/270</v>
+      </c>
+      <c r="D84" t="str">
+        <v>3</v>
+      </c>
+      <c r="E84" t="str">
+        <v>무난</v>
+      </c>
+      <c r="F84" t="str">
+        <v>무난한 디자인이고 무게도 적당. 다만 쿠션감은 조금 아쉽습니다.</v>
+      </c>
+      <c r="G84" t="str">
+        <v>오연재</v>
+      </c>
+      <c r="H84" t="str">
+        <v>2026-05-11</v>
+      </c>
+      <c r="I84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>9008</v>
+      </c>
+      <c r="B85" t="str">
+        <v>러닝화</v>
+      </c>
+      <c r="C85" t="str">
+        <v>블랙/285</v>
+      </c>
+      <c r="D85" t="str">
+        <v>4</v>
+      </c>
+      <c r="E85" t="str">
+        <v>재구매</v>
+      </c>
+      <c r="F85" t="str">
+        <v>발볼만 살짝 좁지만 길들이고 나니 편해요. 색상별로 재구매 의사 있어요.</v>
+      </c>
+      <c r="G85" t="str">
+        <v>신해철</v>
+      </c>
+      <c r="H85" t="str">
+        <v>2026-05-12</v>
+      </c>
+      <c r="I85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>10001</v>
+      </c>
+      <c r="B86" t="str">
+        <v>첼시 부츠</v>
+      </c>
+      <c r="C86" t="str">
+        <v>블랙/265</v>
+      </c>
+      <c r="D86" t="str">
+        <v>3</v>
+      </c>
+      <c r="E86" t="str">
+        <v>사이즈 작음</v>
+      </c>
+      <c r="F86" t="str">
+        <v>평소 사이즈로 샀는데 발볼이 좁고 발가락이 닿아요. 한 치수 크게 권장.</v>
+      </c>
+      <c r="G86" t="str">
+        <v>김민서</v>
+      </c>
+      <c r="H86" t="str">
+        <v>2026-04-18</v>
+      </c>
+      <c r="I86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>10002</v>
+      </c>
+      <c r="B87" t="str">
+        <v>첼시 부츠</v>
+      </c>
+      <c r="C87" t="str">
+        <v>브라운/270</v>
+      </c>
+      <c r="D87" t="str">
+        <v>4</v>
+      </c>
+      <c r="E87" t="str">
+        <v>핏 예뻐요</v>
+      </c>
+      <c r="F87" t="str">
+        <v>발등에 딱 맞고 라인이 예쁩니다. 다만 처음에 뒤꿈치가 살짝 까졌어요.</v>
+      </c>
+      <c r="G87" t="str">
+        <v>이재훈</v>
+      </c>
+      <c r="H87" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="I87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>10003</v>
+      </c>
+      <c r="B88" t="str">
+        <v>첼시 부츠</v>
+      </c>
+      <c r="C88" t="str">
+        <v>블랙/275</v>
+      </c>
+      <c r="D88" t="str">
+        <v>2</v>
+      </c>
+      <c r="E88" t="str">
+        <v>마감 불량</v>
+      </c>
+      <c r="F88" t="str">
+        <v>바닥 본드가 살짝 삐져나와 있고 실밥도 보였어요. 마감이 아쉽네요.</v>
+      </c>
+      <c r="G88" t="str">
+        <v>박세영</v>
+      </c>
+      <c r="H88" t="str">
+        <v>2026-04-20</v>
+      </c>
+      <c r="I88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>10004</v>
+      </c>
+      <c r="B89" t="str">
+        <v>첼시 부츠</v>
+      </c>
+      <c r="C89" t="str">
+        <v>브라운/265</v>
+      </c>
+      <c r="D89" t="str">
+        <v>5</v>
+      </c>
+      <c r="E89" t="str">
+        <v>가성비 좋음</v>
+      </c>
+      <c r="F89" t="str">
+        <v>이 가격에 가죽 마감이 이 정도면 만족합니다. 재구매 의사 있어요.</v>
+      </c>
+      <c r="G89" t="str">
+        <v>최기현</v>
+      </c>
+      <c r="H89" t="str">
+        <v>2026-04-21</v>
+      </c>
+      <c r="I89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>10005</v>
+      </c>
+      <c r="B90" t="str">
+        <v>첼시 부츠</v>
+      </c>
+      <c r="C90" t="str">
+        <v>블랙/270</v>
+      </c>
+      <c r="D90" t="str">
+        <v>3</v>
+      </c>
+      <c r="E90" t="str">
+        <v>길들이는 중</v>
+      </c>
+      <c r="F90" t="str">
+        <v>처음엔 뒤꿈치가 까져서 밴드 필수였는데 길들이니 편해요. 색상은 사진이랑 비슷.</v>
+      </c>
+      <c r="G90" t="str">
+        <v>정승호</v>
+      </c>
+      <c r="H90" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="I90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>10006</v>
+      </c>
+      <c r="B91" t="str">
+        <v>첼시 부츠</v>
+      </c>
+      <c r="C91" t="str">
+        <v>브라운/280</v>
+      </c>
+      <c r="D91" t="str">
+        <v>4</v>
+      </c>
+      <c r="E91" t="str">
+        <v>재구매</v>
+      </c>
+      <c r="F91" t="str">
+        <v>두 켤레째 구매. 발볼은 좁은 편이라 발볼 넓으신 분은 참고하세요.</v>
+      </c>
+      <c r="G91" t="str">
+        <v>한석원</v>
+      </c>
+      <c r="H91" t="str">
+        <v>2026-04-23</v>
+      </c>
+      <c r="I91" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>11001</v>
+      </c>
+      <c r="B92" t="str">
+        <v>숄더백</v>
+      </c>
+      <c r="C92" t="str">
+        <v>블랙/Free</v>
+      </c>
+      <c r="D92" t="str">
+        <v>2</v>
+      </c>
+      <c r="E92" t="str">
+        <v>생각보다 작아요</v>
+      </c>
+      <c r="F92" t="str">
+        <v>사진보다 실물이 작아 보여요. 13인치 노트북이 안 들어가요. 수납공간이 부족합니다.</v>
+      </c>
+      <c r="G92" t="str">
+        <v>김유진</v>
+      </c>
+      <c r="H92" t="str">
+        <v>2026-05-14</v>
+      </c>
+      <c r="I92" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>11002</v>
+      </c>
+      <c r="B93" t="str">
+        <v>숄더백</v>
+      </c>
+      <c r="C93" t="str">
+        <v>베이지/Free</v>
+      </c>
+      <c r="D93" t="str">
+        <v>3</v>
+      </c>
+      <c r="E93" t="str">
+        <v>끈 마감 아쉬움</v>
+      </c>
+      <c r="F93" t="str">
+        <v>끈 박음질이 튀어나와 있고, 가죽 마감도 살짝 거칠어요.</v>
+      </c>
+      <c r="G93" t="str">
+        <v>이수빈</v>
+      </c>
+      <c r="H93" t="str">
+        <v>2026-05-15</v>
+      </c>
+      <c r="I93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>11003</v>
+      </c>
+      <c r="B94" t="str">
+        <v>숄더백</v>
+      </c>
+      <c r="C94" t="str">
+        <v>블랙/Free</v>
+      </c>
+      <c r="D94" t="str">
+        <v>5</v>
+      </c>
+      <c r="E94" t="str">
+        <v>핏 좋아요</v>
+      </c>
+      <c r="F94" t="str">
+        <v>데일리로 메기 좋은 사이즈예요. 색상도 사진이랑 비슷합니다.</v>
+      </c>
+      <c r="G94" t="str">
+        <v>박민지</v>
+      </c>
+      <c r="H94" t="str">
+        <v>2026-05-16</v>
+      </c>
+      <c r="I94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>11004</v>
+      </c>
+      <c r="B95" t="str">
+        <v>숄더백</v>
+      </c>
+      <c r="C95" t="str">
+        <v>브라운/Free</v>
+      </c>
+      <c r="D95" t="str">
+        <v>2</v>
+      </c>
+      <c r="E95" t="str">
+        <v>수납 부족</v>
+      </c>
+      <c r="F95" t="str">
+        <v>파우치 하나 넣으면 꽉 차요. 활용도가 떨어집니다.</v>
+      </c>
+      <c r="G95" t="str">
+        <v>최가은</v>
+      </c>
+      <c r="H95" t="str">
+        <v>2026-05-17</v>
+      </c>
+      <c r="I95" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>11005</v>
+      </c>
+      <c r="B96" t="str">
+        <v>숄더백</v>
+      </c>
+      <c r="C96" t="str">
+        <v>블랙/Free</v>
+      </c>
+      <c r="D96" t="str">
+        <v>3</v>
+      </c>
+      <c r="E96" t="str">
+        <v>포장 구김</v>
+      </c>
+      <c r="F96" t="str">
+        <v>포장 박스가 눌려서 가방이 살짝 구겨져서 왔어요. 다림질로 폈습니다.</v>
+      </c>
+      <c r="G96" t="str">
+        <v>정아영</v>
+      </c>
+      <c r="H96" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="I96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>11006</v>
+      </c>
+      <c r="B97" t="str">
+        <v>숄더백</v>
+      </c>
+      <c r="C97" t="str">
+        <v>베이지/Free</v>
+      </c>
+      <c r="D97" t="str">
+        <v>4</v>
+      </c>
+      <c r="E97" t="str">
+        <v>만족</v>
+      </c>
+      <c r="F97" t="str">
+        <v>예쁘긴 예쁜데 수납이 좀 부족해서 별 하나 뺐어요.</v>
+      </c>
+      <c r="G97" t="str">
+        <v>한채림</v>
+      </c>
+      <c r="H97" t="str">
+        <v>2026-05-19</v>
+      </c>
+      <c r="I97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>12001</v>
+      </c>
+      <c r="B98" t="str">
+        <v>여름 원피스</v>
+      </c>
+      <c r="C98" t="str">
+        <v>화이트/M</v>
+      </c>
+      <c r="D98" t="str">
+        <v>2</v>
+      </c>
+      <c r="E98" t="str">
+        <v>비침 심해요</v>
+      </c>
+      <c r="F98" t="str">
+        <v>원단이 너무 얇아서 비침이 심해요. 속바지 필수입니다.</v>
+      </c>
+      <c r="G98" t="str">
+        <v>김다은</v>
+      </c>
+      <c r="H98" t="str">
+        <v>2026-06-01</v>
+      </c>
+      <c r="I98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>12002</v>
+      </c>
+      <c r="B99" t="str">
+        <v>여름 원피스</v>
+      </c>
+      <c r="C99" t="str">
+        <v>블랙/L</v>
+      </c>
+      <c r="D99" t="str">
+        <v>3</v>
+      </c>
+      <c r="E99" t="str">
+        <v>허리 라인 애매</v>
+      </c>
+      <c r="F99" t="str">
+        <v>허리 라인이 어정쩡해서 핏이 살지 않아요. 색상은 화면이랑 비슷.</v>
+      </c>
+      <c r="G99" t="str">
+        <v>이연우</v>
+      </c>
+      <c r="H99" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="I99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>12003</v>
+      </c>
+      <c r="B100" t="str">
+        <v>여름 원피스</v>
+      </c>
+      <c r="C100" t="str">
+        <v>네이비/M</v>
+      </c>
+      <c r="D100" t="str">
+        <v>2</v>
+      </c>
+      <c r="E100" t="str">
+        <v>기장이 너무 김</v>
+      </c>
+      <c r="F100" t="str">
+        <v>키 165인데 발목까지 와요. 단 수선이 필요했어요.</v>
+      </c>
+      <c r="G100" t="str">
+        <v>박서연</v>
+      </c>
+      <c r="H100" t="str">
+        <v>2026-06-03</v>
+      </c>
+      <c r="I100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>12004</v>
+      </c>
+      <c r="B101" t="str">
+        <v>여름 원피스</v>
+      </c>
+      <c r="C101" t="str">
+        <v>화이트/S</v>
+      </c>
+      <c r="D101" t="str">
+        <v>5</v>
+      </c>
+      <c r="E101" t="str">
+        <v>시원해요</v>
+      </c>
+      <c r="F101" t="str">
+        <v>여름에 입기 시원하고 핏도 예뻐요. 비침은 약간 있지만 만족.</v>
+      </c>
+      <c r="G101" t="str">
+        <v>최지윤</v>
+      </c>
+      <c r="H101" t="str">
+        <v>2026-06-04</v>
+      </c>
+      <c r="I101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>12005</v>
+      </c>
+      <c r="B102" t="str">
+        <v>여름 원피스</v>
+      </c>
+      <c r="C102" t="str">
+        <v>블랙/M</v>
+      </c>
+      <c r="D102" t="str">
+        <v>3</v>
+      </c>
+      <c r="E102" t="str">
+        <v>무난</v>
+      </c>
+      <c r="F102" t="str">
+        <v>무난한 디자인. 다만 원단이 살짝 얇은 편이라 이너 추천.</v>
+      </c>
+      <c r="G102" t="str">
+        <v>정우진</v>
+      </c>
+      <c r="H102" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="I102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>12006</v>
+      </c>
+      <c r="B103" t="str">
+        <v>여름 원피스</v>
+      </c>
+      <c r="C103" t="str">
+        <v>네이비/L</v>
+      </c>
+      <c r="D103" t="str">
+        <v>4</v>
+      </c>
+      <c r="E103" t="str">
+        <v>재구매 의사</v>
+      </c>
+      <c r="F103" t="str">
+        <v>색상별로 사고 싶을 만큼 예뻐요. 비침만 보완되면 더 좋겠어요.</v>
+      </c>
+      <c r="G103" t="str">
+        <v>한소연</v>
+      </c>
+      <c r="H103" t="str">
+        <v>2026-06-06</v>
+      </c>
+      <c r="I103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>13001</v>
+      </c>
+      <c r="B104" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C104" t="str">
+        <v>아이보리/Free</v>
+      </c>
+      <c r="D104" t="str">
+        <v>2</v>
+      </c>
+      <c r="E104" t="str">
+        <v>어깨가 좁아요</v>
+      </c>
+      <c r="F104" t="str">
+        <v>어깨가 너무 좁아서 답답해요. 핏이 예쁘다고 해서 샀는데 좀 아쉬워요.</v>
+      </c>
+      <c r="G104" t="str">
+        <v>김도아</v>
+      </c>
+      <c r="H104" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="I104" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>13002</v>
+      </c>
+      <c r="B105" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C105" t="str">
+        <v>블랙/Free</v>
+      </c>
+      <c r="D105" t="str">
+        <v>2</v>
+      </c>
+      <c r="E105" t="str">
+        <v>보풀 잘 생겨요</v>
+      </c>
+      <c r="F105" t="str">
+        <v>한 번 입었는데 보풀이 잔뜩 생겼어요. 내구성이 약합니다.</v>
+      </c>
+      <c r="G105" t="str">
+        <v>이수아</v>
+      </c>
+      <c r="H105" t="str">
+        <v>2026-04-06</v>
+      </c>
+      <c r="I105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>13003</v>
+      </c>
+      <c r="B106" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C106" t="str">
+        <v>베이지/Free</v>
+      </c>
+      <c r="D106" t="str">
+        <v>5</v>
+      </c>
+      <c r="E106" t="str">
+        <v>따뜻하고 예뻐요</v>
+      </c>
+      <c r="F106" t="str">
+        <v>크롭 길이도 적당하고 부드러워요. 색상별로 사고 싶을 정도예요.</v>
+      </c>
+      <c r="G106" t="str">
+        <v>박혜린</v>
+      </c>
+      <c r="H106" t="str">
+        <v>2026-04-07</v>
+      </c>
+      <c r="I106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>13004</v>
+      </c>
+      <c r="B107" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C107" t="str">
+        <v>아이보리/Free</v>
+      </c>
+      <c r="D107" t="str">
+        <v>3</v>
+      </c>
+      <c r="E107" t="str">
+        <v>비침 살짝</v>
+      </c>
+      <c r="F107" t="str">
+        <v>얇은 편이라 살짝 비쳐요. 이너 필수입니다. 색상은 사진이랑 비슷.</v>
+      </c>
+      <c r="G107" t="str">
+        <v>최서진</v>
+      </c>
+      <c r="H107" t="str">
+        <v>2026-04-08</v>
+      </c>
+      <c r="I107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>13005</v>
+      </c>
+      <c r="B108" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C108" t="str">
+        <v>차콜/Free</v>
+      </c>
+      <c r="D108" t="str">
+        <v>2</v>
+      </c>
+      <c r="E108" t="str">
+        <v>세탁 후 변형</v>
+      </c>
+      <c r="F108" t="str">
+        <v>드라이만 했는데 어깨 라인이 틀어졌어요. 세탁 주의가 필요해 보여요. 문의는 010-9876-5432.</v>
+      </c>
+      <c r="G108" t="str">
+        <v>정우림</v>
+      </c>
+      <c r="H108" t="str">
+        <v>2026-04-09</v>
+      </c>
+      <c r="I108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>13006</v>
+      </c>
+      <c r="B109" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C109" t="str">
+        <v>블랙/Free</v>
+      </c>
+      <c r="D109" t="str">
+        <v>4</v>
+      </c>
+      <c r="E109" t="str">
+        <v>재구매 의사</v>
+      </c>
+      <c r="F109" t="str">
+        <v>핏이 예쁘게 떨어져요. 다만 보풀이 좀 생기네요. 그래도 만족.</v>
+      </c>
+      <c r="G109" t="str">
+        <v>한지수</v>
+      </c>
+      <c r="H109" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="I109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>13007</v>
+      </c>
+      <c r="B110" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C110" t="str">
+        <v>베이지/Free</v>
+      </c>
+      <c r="D110" t="str">
+        <v>3</v>
+      </c>
+      <c r="E110" t="str">
+        <v>냄새</v>
+      </c>
+      <c r="F110" t="str">
+        <v>새 제품 특유의 냄새가 좀 났어요. 며칠 환기하니 괜찮아졌어요.</v>
+      </c>
+      <c r="G110" t="str">
+        <v>오민지</v>
+      </c>
+      <c r="H110" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="I110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>14001</v>
+      </c>
+      <c r="B111" t="str">
+        <v>코튼 조거팬츠</v>
+      </c>
+      <c r="C111" t="str">
+        <v>블랙/M</v>
+      </c>
+      <c r="D111" t="str">
+        <v>4</v>
+      </c>
+      <c r="E111" t="str">
+        <v>편해요</v>
+      </c>
+      <c r="F111" t="str">
+        <v>착용감이 편하고 핏도 좋아요. 색상도 사진이랑 비슷합니다. 가성비 굿.</v>
+      </c>
+      <c r="G111" t="str">
+        <v>김태우</v>
+      </c>
+      <c r="H111" t="str">
+        <v>2026-05-25</v>
+      </c>
+      <c r="I111" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>14002</v>
+      </c>
+      <c r="B112" t="str">
+        <v>코튼 조거팬츠</v>
+      </c>
+      <c r="C112" t="str">
+        <v>그레이/L</v>
+      </c>
+      <c r="D112" t="str">
+        <v>2</v>
+      </c>
+      <c r="E112" t="str">
+        <v>사이즈 작음</v>
+      </c>
+      <c r="F112" t="str">
+        <v>평소 사이즈 샀는데 허리가 살짝 끼고 기장이 짧아요. 한 치수 크게 권장.</v>
+      </c>
+      <c r="G112" t="str">
+        <v>이현수</v>
+      </c>
+      <c r="H112" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="I112" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>14003</v>
+      </c>
+      <c r="B113" t="str">
+        <v>코튼 조거팬츠</v>
+      </c>
+      <c r="C113" t="str">
+        <v>블랙/L</v>
+      </c>
+      <c r="D113" t="str">
+        <v>3</v>
+      </c>
+      <c r="E113" t="str">
+        <v>색상 차이</v>
+      </c>
+      <c r="F113" t="str">
+        <v>블랙인데 실물은 짙은 차콜에 가까워요. 톤이 좀 달라요.</v>
+      </c>
+      <c r="G113" t="str">
+        <v>박지훈</v>
+      </c>
+      <c r="H113" t="str">
+        <v>2026-05-27</v>
+      </c>
+      <c r="I113" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>14004</v>
+      </c>
+      <c r="B114" t="str">
+        <v>코튼 조거팬츠</v>
+      </c>
+      <c r="C114" t="str">
+        <v>그레이/M</v>
+      </c>
+      <c r="D114" t="str">
+        <v>5</v>
+      </c>
+      <c r="E114" t="str">
+        <v>재구매</v>
+      </c>
+      <c r="F114" t="str">
+        <v>두 켤레째 구매. 가성비 정말 좋아요. 색상별로 살 예정입니다.</v>
+      </c>
+      <c r="G114" t="str">
+        <v>최민수</v>
+      </c>
+      <c r="H114" t="str">
+        <v>2026-05-28</v>
+      </c>
+      <c r="I114" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>14005</v>
+      </c>
+      <c r="B115" t="str">
+        <v>코튼 조거팬츠</v>
+      </c>
+      <c r="C115" t="str">
+        <v>네이비/L</v>
+      </c>
+      <c r="D115" t="str">
+        <v>2</v>
+      </c>
+      <c r="E115" t="str">
+        <v>밴딩 헐거움</v>
+      </c>
+      <c r="F115" t="str">
+        <v>허리 밴딩이 헐거워서 자꾸 내려와요. 사이즈 조절이 어려워요.</v>
+      </c>
+      <c r="G115" t="str">
+        <v>정은채</v>
+      </c>
+      <c r="H115" t="str">
+        <v>2026-05-29</v>
+      </c>
+      <c r="I115" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>14006</v>
+      </c>
+      <c r="B116" t="str">
+        <v>코튼 조거팬츠</v>
+      </c>
+      <c r="C116" t="str">
+        <v>블랙/M</v>
+      </c>
+      <c r="D116" t="str">
+        <v>3</v>
+      </c>
+      <c r="E116" t="str">
+        <v>세탁 후 줄어듦</v>
+      </c>
+      <c r="F116" t="str">
+        <v>한 번 세탁했는데 기장이 살짝 줄었어요. 처음엔 적당했는데.</v>
+      </c>
+      <c r="G116" t="str">
+        <v>한상우</v>
+      </c>
+      <c r="H116" t="str">
+        <v>2026-05-30</v>
+      </c>
+      <c r="I116" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>14007</v>
+      </c>
+      <c r="B117" t="str">
+        <v>코튼 조거팬츠</v>
+      </c>
+      <c r="C117" t="str">
+        <v>그레이/L</v>
+      </c>
+      <c r="D117" t="str">
+        <v>4</v>
+      </c>
+      <c r="E117" t="str">
+        <v>만족</v>
+      </c>
+      <c r="F117" t="str">
+        <v>편하게 입기 좋아요. 다만 무릎 부분이 금방 늘어나는 느낌.</v>
+      </c>
+      <c r="G117" t="str">
+        <v>오지영</v>
+      </c>
+      <c r="H117" t="str">
+        <v>2026-05-31</v>
+      </c>
+      <c r="I117" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>15001</v>
+      </c>
+      <c r="B118" t="str">
+        <v>슬림핏 셔츠</v>
+      </c>
+      <c r="C118" t="str">
+        <v>화이트/M</v>
+      </c>
+      <c r="D118" t="str">
+        <v>4</v>
+      </c>
+      <c r="E118" t="str">
+        <v>데일리하게 입기 좋아요</v>
+      </c>
+      <c r="F118" t="str">
+        <v>핏은 예쁜데 기장이 제 기준에는 살짝 길어요. 그래도 데일리로 입기 무난합니다.</v>
+      </c>
+      <c r="G118" t="str">
+        <v>박서연</v>
+      </c>
+      <c r="H118" t="str">
+        <v>2026-06-01</v>
+      </c>
+      <c r="I118" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>15002</v>
+      </c>
+      <c r="B119" t="str">
+        <v>슬림핏 셔츠</v>
+      </c>
+      <c r="C119" t="str">
+        <v>블루/L</v>
+      </c>
+      <c r="D119" t="str">
+        <v>4</v>
+      </c>
+      <c r="E119" t="str">
+        <v>어깨가 조금 큼</v>
+      </c>
+      <c r="F119" t="str">
+        <v>기장은 괜찮은데 어깨가 조금 크게 느껴져요. 마감이 나쁘지 않아서 오래 입을 수 있을 것 같아요.</v>
+      </c>
+      <c r="G119" t="str">
+        <v>이지원</v>
+      </c>
+      <c r="H119" t="str">
+        <v>2026-06-01</v>
+      </c>
+      <c r="I119" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>15003</v>
+      </c>
+      <c r="B120" t="str">
+        <v>오버핏 반팔 티셔츠</v>
+      </c>
+      <c r="C120" t="str">
+        <v>화이트/L</v>
+      </c>
+      <c r="D120" t="str">
+        <v>5</v>
+      </c>
+      <c r="E120" t="str">
+        <v>비침 걱정 없음</v>
+      </c>
+      <c r="F120" t="str">
+        <v>화이트인데도 비침이 거의 없어서 만족합니다. 원단도 탄탄해서 좋아요.</v>
+      </c>
+      <c r="G120" t="str">
+        <v>김도윤</v>
+      </c>
+      <c r="H120" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="I120" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>15004</v>
+      </c>
+      <c r="B121" t="str">
+        <v>오버핏 반팔 티셔츠</v>
+      </c>
+      <c r="C121" t="str">
+        <v>그레이/M</v>
+      </c>
+      <c r="D121" t="str">
+        <v>3</v>
+      </c>
+      <c r="E121" t="str">
+        <v>사이즈 다운 추천</v>
+      </c>
+      <c r="F121" t="str">
+        <v>생각보다 품이 커서 정핏을 원하면 한 치수 작게 사는 게 좋겠어요. 색상은 사진과 비슷합니다.</v>
+      </c>
+      <c r="G121" t="str">
+        <v>조하늘</v>
+      </c>
+      <c r="H121" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="I121" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>15005</v>
+      </c>
+      <c r="B122" t="str">
+        <v>여름 원피스</v>
+      </c>
+      <c r="C122" t="str">
+        <v>핑크/S</v>
+      </c>
+      <c r="D122" t="str">
+        <v>4</v>
+      </c>
+      <c r="E122" t="str">
+        <v>색감 차이 약간</v>
+      </c>
+      <c r="F122" t="str">
+        <v>사진보다 색감이 조금 밝게 느껴졌어요. 가격 생각하면 충분히 만족스러운 편입니다.</v>
+      </c>
+      <c r="G122" t="str">
+        <v>윤서아</v>
+      </c>
+      <c r="H122" t="str">
+        <v>2026-06-03</v>
+      </c>
+      <c r="I122" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>15006</v>
+      </c>
+      <c r="B123" t="str">
+        <v>여름 원피스</v>
+      </c>
+      <c r="C123" t="str">
+        <v>블랙/M</v>
+      </c>
+      <c r="D123" t="str">
+        <v>2</v>
+      </c>
+      <c r="E123" t="str">
+        <v>색감 차이</v>
+      </c>
+      <c r="F123" t="str">
+        <v>사진보다 실물이 더 어두워요. 색상 차이가 조금 있습니다.</v>
+      </c>
+      <c r="G123" t="str">
+        <v>한가람</v>
+      </c>
+      <c r="H123" t="str">
+        <v>2026-06-03</v>
+      </c>
+      <c r="I123" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>15007</v>
+      </c>
+      <c r="B124" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C124" t="str">
+        <v>베이지/L</v>
+      </c>
+      <c r="D124" t="str">
+        <v>5</v>
+      </c>
+      <c r="E124" t="str">
+        <v>재구매 의사</v>
+      </c>
+      <c r="F124" t="str">
+        <v>가격 대비 품질이 좋아서 색상별로 더 사고 싶어요. 마감이 나쁘지 않아서 오래 입을 수 있을 것 같아요.</v>
+      </c>
+      <c r="G124" t="str">
+        <v>장수빈</v>
+      </c>
+      <c r="H124" t="str">
+        <v>2026-06-04</v>
+      </c>
+      <c r="I124" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>15008</v>
+      </c>
+      <c r="B125" t="str">
+        <v>트렌치 코트</v>
+      </c>
+      <c r="C125" t="str">
+        <v>블랙/M</v>
+      </c>
+      <c r="D125" t="str">
+        <v>4</v>
+      </c>
+      <c r="E125" t="str">
+        <v>재질 만족</v>
+      </c>
+      <c r="F125" t="str">
+        <v>재질은 괜찮은데 생각보다 두꺼워서 한여름에는 조금 더울 수 있어요.</v>
+      </c>
+      <c r="G125" t="str">
+        <v>서지호</v>
+      </c>
+      <c r="H125" t="str">
+        <v>2026-06-04</v>
+      </c>
+      <c r="I125" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>15009</v>
+      </c>
+      <c r="B126" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C126" t="str">
+        <v>화이트/M</v>
+      </c>
+      <c r="D126" t="str">
+        <v>5</v>
+      </c>
+      <c r="E126" t="str">
+        <v>세탁 후에도 그대로</v>
+      </c>
+      <c r="F126" t="str">
+        <v>세탁 후에도 크게 줄어들지 않았어요. 가격 대비 만족합니다.</v>
+      </c>
+      <c r="G126" t="str">
+        <v>임채원</v>
+      </c>
+      <c r="H126" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="I126" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>15010</v>
+      </c>
+      <c r="B127" t="str">
+        <v>크롭 니트</v>
+      </c>
+      <c r="C127" t="str">
+        <v>베이지/L</v>
+      </c>
+      <c r="D127" t="str">
+        <v>2</v>
+      </c>
+      <c r="E127" t="str">
+        <v>비침 심함</v>
+      </c>
+      <c r="F127" t="str">
+        <v>화이트 색상은 속옷이 비쳐서 단독으로 입기 어려워요. 이너 필수입니다.</v>
+      </c>
+      <c r="G127" t="str">
+        <v>강민주</v>
+      </c>
+      <c r="H127" t="str">
+        <v>2026-06-05</v>
+      </c>
+      <c r="I127" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>15011</v>
+      </c>
+      <c r="B128" t="str">
+        <v>니트 가디건</v>
+      </c>
+      <c r="C128" t="str">
+        <v>그레이/M</v>
+      </c>
+      <c r="D128" t="str">
+        <v>3</v>
+      </c>
+      <c r="E128" t="str">
+        <v>마감 아쉬움</v>
+      </c>
+      <c r="F128" t="str">
+        <v>박음질이 조금 삐뚤고 실밥이 몇 군데 보여요. 가격 대비 품질이 아쉬워요.</v>
+      </c>
+      <c r="G128" t="str">
+        <v>노유진</v>
+      </c>
+      <c r="H128" t="str">
+        <v>2026-06-06</v>
+      </c>
+      <c r="I128" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>15012</v>
+      </c>
+      <c r="B129" t="str">
+        <v>니트 가디건</v>
+      </c>
+      <c r="C129" t="str">
+        <v>네이비/L</v>
+      </c>
+      <c r="D129" t="str">
+        <v>5</v>
+      </c>
+      <c r="E129" t="str">
+        <v>마감 깔끔</v>
+      </c>
+      <c r="F129" t="str">
+        <v>실밥 없이 마감이 깔끔해서 만족합니다. 박음질도 꼼꼼해요.</v>
+      </c>
+      <c r="G129" t="str">
+        <v>김태현</v>
+      </c>
+      <c r="H129" t="str">
+        <v>2026-06-06</v>
+      </c>
+      <c r="I129" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>15013</v>
+      </c>
+      <c r="B130" t="str">
+        <v>첼시 부츠</v>
+      </c>
+      <c r="C130" t="str">
+        <v>블랙/240</v>
+      </c>
+      <c r="D130" t="str">
+        <v>2</v>
+      </c>
+      <c r="E130" t="str">
+        <v>발볼이 좁아요</v>
+      </c>
+      <c r="F130" t="str">
+        <v>발볼이 좁아서 오래 걸으면 발이 아파요. 한 치수 크게 주문하시는 걸 추천드려요.</v>
+      </c>
+      <c r="G130" t="str">
+        <v>정혜원</v>
+      </c>
+      <c r="H130" t="str">
+        <v>2026-06-07</v>
+      </c>
+      <c r="I130" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>15014</v>
+      </c>
+      <c r="B131" t="str">
+        <v>첼시 부츠</v>
+      </c>
+      <c r="C131" t="str">
+        <v>브라운/250</v>
+      </c>
+      <c r="D131" t="str">
+        <v>5</v>
+      </c>
+      <c r="E131" t="str">
+        <v>배송과 포장 만족</v>
+      </c>
+      <c r="F131" t="str">
+        <v>배송도 빠르고 포장도 깔끔했어요. 옷장에 잘 보관하고 잘 신고 있습니다.</v>
+      </c>
+      <c r="G131" t="str">
+        <v>이준호</v>
+      </c>
+      <c r="H131" t="str">
+        <v>2026-06-07</v>
+      </c>
+      <c r="I131" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>15015</v>
+      </c>
+      <c r="B132" t="str">
+        <v>플리츠 롱스커트</v>
+      </c>
+      <c r="C132" t="str">
+        <v>그레이/S</v>
+      </c>
+      <c r="D132" t="str">
+        <v>3</v>
+      </c>
+      <c r="E132" t="str">
+        <v>포장 구김</v>
+      </c>
+      <c r="F132" t="str">
+        <v>배송은 빨랐지만 포장이 구겨져서 옷에 주름이 많이 생겼어요.</v>
+      </c>
+      <c r="G132" t="str">
+        <v>오세린</v>
+      </c>
+      <c r="H132" t="str">
+        <v>2026-06-08</v>
+      </c>
+      <c r="I132" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>15016</v>
+      </c>
+      <c r="B133" t="str">
+        <v>오버핏 후드 집업</v>
+      </c>
+      <c r="C133" t="str">
+        <v>블랙/L</v>
+      </c>
+      <c r="D133" t="str">
+        <v>4</v>
+      </c>
+      <c r="E133" t="str">
+        <v>목 부분 살짝 타이트</v>
+      </c>
+      <c r="F133" t="str">
+        <v>목 부분이 조금 타이트하게 느껴졌지만 입다 보면 괜찮을 것 같습니다.</v>
+      </c>
+      <c r="G133" t="str">
+        <v>박지민</v>
+      </c>
+      <c r="H133" t="str">
+        <v>2026-06-09</v>
+      </c>
+      <c r="I133" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>15017</v>
+      </c>
+      <c r="B134" t="str">
+        <v>슬림핏 셔츠</v>
+      </c>
+      <c r="C134" t="str">
+        <v>블루/M</v>
+      </c>
+      <c r="D134" t="str">
+        <v>3</v>
+      </c>
+      <c r="E134" t="str">
+        <v>허리 타이트</v>
+      </c>
+      <c r="F134" t="str">
+        <v>기장은 괜찮고 허리가 조금 타이트해요. 한 치수 크게 사시는 게 나을 듯합니다.</v>
+      </c>
+      <c r="G134" t="str">
+        <v>홍은서</v>
+      </c>
+      <c r="H134" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="I134" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I134"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>사례</v>
+      </c>
+      <c r="B1" t="str">
+        <v>리뷰내용</v>
+      </c>
+      <c r="C1" t="str">
+        <v>기대결과</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>긍정</v>
+      </c>
+      <c r="B2" t="str">
+        <v>가격 대비 품질이 좋아서 색상별로 더 사고 싶어요.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>actionable 없음</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>대조</v>
+      </c>
+      <c r="B3" t="str">
+        <v>기장은 괜찮은데 어깨가 조금 크게 느껴져요.</v>
+      </c>
+      <c r="C3" t="str">
+        <v>어깨가 큼만</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>방향성</v>
+      </c>
+      <c r="B4" t="str">
+        <v>품이 커서 한 치수 작게 사세요.</v>
+      </c>
+      <c r="C4" t="str">
+        <v>전반적으로 크게 나옴</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>지표</v>
+      </c>
+      <c r="B1" t="str">
+        <v>값</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>총 리뷰 수</v>
+      </c>
+      <c r="B2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>주요 상품군</v>
+      </c>
+      <c r="B3" t="str">
+        <v>의류·신발·가방</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>리뷰핏 샘플 데이터</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>아래 데이터는 테스트용입니다. 실제 셀러 데이터가 아닙니다.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>시트 구성: 리뷰데이터 / 오분류_테스트케이스 / 요약 / README</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>